<commit_message>
Rerun Conformist to double check errors
</commit_message>
<xml_diff>
--- a/data/conf_ta_output/conf_ta_tw.xlsx
+++ b/data/conf_ta_output/conf_ta_tw.xlsx
@@ -136,13 +136,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -376,340 +380,352 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C2" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E2" s="0" t="n">
+      <c r="A2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E2" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H2" s="0" t="n">
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>0.0588235294117647</v>
       </c>
-      <c r="I2" s="0" t="n">
+      <c r="I2" s="2" t="n">
         <v>0.941176470588235</v>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="J2" s="2" t="n">
         <v>0.949</v>
       </c>
-      <c r="K2" s="0" t="n">
+      <c r="K2" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B3" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C3" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E3" s="0" t="n">
+      <c r="A3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="0" t="n">
+      <c r="G3" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="n">
         <v>0.085</v>
       </c>
-      <c r="K3" s="0" t="n">
+      <c r="K3" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C4" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E4" s="0" t="n">
+      <c r="A4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G4" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H4" s="0" t="n">
+      <c r="G4" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>0.00105042016806723</v>
       </c>
-      <c r="I4" s="0" t="n">
+      <c r="I4" s="2" t="n">
         <v>0.998949579831933</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="2" t="n">
         <v>0.048</v>
       </c>
-      <c r="K4" s="0" t="n">
+      <c r="K4" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C5" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E5" s="0" t="n">
+      <c r="A5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G5" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="J5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="0" t="n">
+      <c r="G5" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E6" s="0" t="n">
+      <c r="A6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="F6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="0" t="n">
+      <c r="F6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>0.958</v>
       </c>
-      <c r="K6" s="0" t="n">
+      <c r="K6" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C7" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E7" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F7" s="0" t="n">
+      <c r="A7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H7" s="0" t="n">
+      <c r="G7" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>0.0444444444444445</v>
       </c>
-      <c r="I7" s="0" t="n">
+      <c r="I7" s="2" t="n">
         <v>0.955555555555556</v>
       </c>
-      <c r="J7" s="0" t="n">
+      <c r="J7" s="2" t="n">
         <v>0.955</v>
       </c>
-      <c r="K7" s="0" t="n">
+      <c r="K7" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C8" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E8" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="0" t="n">
+      <c r="A8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G8" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H8" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="0" t="n">
+      <c r="G8" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2" t="n">
         <v>0.14</v>
       </c>
-      <c r="K8" s="0" t="n">
+      <c r="K8" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C9" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D9" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E9" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F9" s="0" t="n">
+      <c r="A9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="G9" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="0" t="n">
+      <c r="G9" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2" t="n">
         <v>0.049</v>
       </c>
-      <c r="K9" s="0" t="n">
+      <c r="K9" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C10" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D10" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E10" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F10" s="0" t="n">
+      <c r="A10" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G10" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H10" s="0" t="n">
+      <c r="G10" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>0.0031413612565445</v>
       </c>
-      <c r="I10" s="0" t="n">
+      <c r="I10" s="2" t="n">
         <v>0.996858638743456</v>
       </c>
-      <c r="J10" s="0" t="n">
+      <c r="J10" s="2" t="n">
         <v>0.045</v>
       </c>
-      <c r="K10" s="0" t="n">
+      <c r="K10" s="2" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C11" s="0" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D11" s="0" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E11" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F11" s="0" t="n">
+      <c r="A11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G11" s="0" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="J11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="0" t="n">
+      <c r="G11" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="n">
         <v>1000</v>
       </c>
     </row>

</xml_diff>